<commit_message>
feat: add 7-day free trial with 10 SMS limit
- Add TRIAL_SMS_LIMIT constant (10 requests)
- Add isTrialActive and trialEndsAt fields to BusinessProfile
- Edge function enforces trial limit before tier quota
- Trial-specific error message directs to subscription page
- Dashboard quota warning and settings usage bar are trial-aware
- DB migration needed: is_trial_active BOOLEAN, trial_ends_at TIMESTAMPTZ
</commit_message>
<xml_diff>
--- a/scripts/leads-master.xlsx
+++ b/scripts/leads-master.xlsx
@@ -6,6 +6,9 @@
     <sheet name="Batch 1" sheetId="1" r:id="rId1"/>
     <sheet name="Batch 2" sheetId="2" r:id="rId2"/>
     <sheet name="Batch 3" sheetId="3" r:id="rId3"/>
+    <sheet name="Batch 4" sheetId="4" r:id="rId4"/>
+    <sheet name="Batch 5" sheetId="5" r:id="rId5"/>
+    <sheet name="Batch 6" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -400,17 +403,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I26"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="35.83203125" customWidth="1"/>
-    <col min="3" max="3" width="6.83203125" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="40.83203125" customWidth="1"/>
-    <col min="7" max="7" width="50.83203125" customWidth="1"/>
-    <col min="8" max="8" width="45.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1176,17 +1168,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I26"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="35.83203125" customWidth="1"/>
-    <col min="3" max="3" width="6.83203125" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="40.83203125" customWidth="1"/>
-    <col min="7" max="7" width="50.83203125" customWidth="1"/>
-    <col min="8" max="8" width="45.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1952,15 +1933,1168 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I19"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Business Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Stars</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Reviews</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Website</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Google Maps URL</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Address</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Date Found</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Bryan Electric, Inc.</v>
+      </c>
+      <c r="B2" t="str">
+        <v>info@bryanelectricinc.com</v>
+      </c>
+      <c r="C2" t="str">
+        <v>4</v>
+      </c>
+      <c r="D2" t="str">
+        <v>21</v>
+      </c>
+      <c r="E2" t="str">
+        <v>(770) 680-2144</v>
+      </c>
+      <c r="F2" t="str">
+        <v>http://www.bryanelectricinc.com/</v>
+      </c>
+      <c r="G2" t="str">
+        <v>https://maps.google.com/?cid=14552314039426656722&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H2" t="str">
+        <v>1840 Grassland Pkwy #200, Alpharetta, GA 30004, USA</v>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>JustFixToday - Handyman Services in Alpharetta GA | Painter | Plumber | Drywall | AC Repair | Electrical Repair | Carpenter</v>
+      </c>
+      <c r="B3" t="str">
+        <v>info@justfixtoday.com</v>
+      </c>
+      <c r="C3" t="str">
+        <v>5</v>
+      </c>
+      <c r="D3" t="str">
+        <v>135</v>
+      </c>
+      <c r="E3" t="str">
+        <v>(678) 549-8083</v>
+      </c>
+      <c r="F3" t="str">
+        <v>https://www.justfixtoday.com/</v>
+      </c>
+      <c r="G3" t="str">
+        <v>https://maps.google.com/?cid=1787476070147627322&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H3" t="str">
+        <v>2425 Traywick Chase, Alpharetta, GA 30004, USA</v>
+      </c>
+      <c r="I3" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Southern Electric Co</v>
+      </c>
+      <c r="B4" t="str">
+        <v>controller@southernelectriccompany.com</v>
+      </c>
+      <c r="C4" t="str">
+        <v>4.2</v>
+      </c>
+      <c r="D4" t="str">
+        <v>11</v>
+      </c>
+      <c r="E4" t="str">
+        <v>(770) 740-9553</v>
+      </c>
+      <c r="F4" t="str">
+        <v>https://southernelectriccompany.com/</v>
+      </c>
+      <c r="G4" t="str">
+        <v>https://maps.google.com/?cid=2412617203072986788&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H4" t="str">
+        <v>510 Winkler Dr #100, Alpharetta, GA 30004, USA</v>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Sharp Electrical Contractors</v>
+      </c>
+      <c r="B5" t="str">
+        <v>impallari@gmail.com</v>
+      </c>
+      <c r="C5" t="str">
+        <v>5</v>
+      </c>
+      <c r="D5" t="str">
+        <v>12</v>
+      </c>
+      <c r="E5" t="str">
+        <v>(678) 939-1907</v>
+      </c>
+      <c r="F5" t="str">
+        <v>http://www.sharpelectricalcontractorsinc.com/</v>
+      </c>
+      <c r="G5" t="str">
+        <v>https://maps.google.com/?cid=15784420237876544597&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H5" t="str">
+        <v>4571 Oakhurst Ln, Alpharetta, GA 30004, USA</v>
+      </c>
+      <c r="I5" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Ray's Electrical Services, LLC.</v>
+      </c>
+      <c r="B6" t="str">
+        <v>ray.electric@yahoo.com</v>
+      </c>
+      <c r="C6" t="str">
+        <v>5</v>
+      </c>
+      <c r="D6" t="str">
+        <v>33</v>
+      </c>
+      <c r="E6" t="str">
+        <v>(404) 934-3725</v>
+      </c>
+      <c r="F6" t="str">
+        <v>https://rayselectricalservices.net/</v>
+      </c>
+      <c r="G6" t="str">
+        <v>https://maps.google.com/?cid=17255572914718368004&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H6" t="str">
+        <v>11877 Douglas Rd, Johns Creek, GA 30005, USA</v>
+      </c>
+      <c r="I6" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>JA IT ELECTRIC</v>
+      </c>
+      <c r="B7" t="str">
+        <v>contact@jaitelectric.com</v>
+      </c>
+      <c r="C7" t="str">
+        <v>4.9</v>
+      </c>
+      <c r="D7" t="str">
+        <v>79</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>https://www.jaitelectric.com/</v>
+      </c>
+      <c r="G7" t="str">
+        <v>https://maps.google.com/?cid=16789752584030982869&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H7" t="str">
+        <v>3824 Dandridge Way NW, Duluth, GA 30096, USA</v>
+      </c>
+      <c r="I7" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>DSL Electric</v>
+      </c>
+      <c r="B8" t="str">
+        <v>dslelectric@yahoo.com</v>
+      </c>
+      <c r="C8" t="str">
+        <v>4.7</v>
+      </c>
+      <c r="D8" t="str">
+        <v>143</v>
+      </c>
+      <c r="E8" t="str">
+        <v>(470) 637-2322</v>
+      </c>
+      <c r="F8" t="str">
+        <v>https://www.dslelectric.net/</v>
+      </c>
+      <c r="G8" t="str">
+        <v>https://maps.google.com/?cid=1906140520379199906&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H8" t="str">
+        <v>1159 Reading Dr NW, Acworth, GA 30102, USA</v>
+      </c>
+      <c r="I8" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>M.D. Contracting Solutions</v>
+      </c>
+      <c r="B9" t="str">
+        <v>admin@mdcontractingsolutions.com</v>
+      </c>
+      <c r="C9" t="str">
+        <v>5</v>
+      </c>
+      <c r="D9" t="str">
+        <v>137</v>
+      </c>
+      <c r="E9" t="str">
+        <v>(678) 636-9692</v>
+      </c>
+      <c r="F9" t="str">
+        <v>https://www.mdcontractingsolutions.com/</v>
+      </c>
+      <c r="G9" t="str">
+        <v>https://maps.google.com/?cid=9302632286792896560&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H9" t="str">
+        <v>2244 NW Pkwy SE Ste A, Marietta, GA 30067, USA</v>
+      </c>
+      <c r="I9" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>VIP Electrical Service</v>
+      </c>
+      <c r="B10" t="str">
+        <v>vipelservice@gmail.com</v>
+      </c>
+      <c r="C10" t="str">
+        <v>5</v>
+      </c>
+      <c r="D10" t="str">
+        <v>57</v>
+      </c>
+      <c r="E10" t="str">
+        <v>(706) 510-5132</v>
+      </c>
+      <c r="F10" t="str">
+        <v>http://vipelectricalservice.co/</v>
+      </c>
+      <c r="G10" t="str">
+        <v>https://maps.google.com/?cid=5752995803636552844&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H10" t="str">
+        <v>3327 Club Pl, Duluth, GA 30096, USA</v>
+      </c>
+      <c r="I10" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Alpine Electrical Solutions</v>
+      </c>
+      <c r="B11" t="str">
+        <v>info@alpelecsolutions.com</v>
+      </c>
+      <c r="C11" t="str">
+        <v>5</v>
+      </c>
+      <c r="D11" t="str">
+        <v>14</v>
+      </c>
+      <c r="E11" t="str">
+        <v>(470) 896-6060</v>
+      </c>
+      <c r="F11" t="str">
+        <v>https://alpelecsolutions.com/</v>
+      </c>
+      <c r="G11" t="str">
+        <v>https://maps.google.com/?cid=5558601400349421621&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H11" t="str">
+        <v>3675 Crestwood Pkwy NW #400, Duluth, GA 30096, USA</v>
+      </c>
+      <c r="I11" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>GE Martin Electrical LLC</v>
+      </c>
+      <c r="B12" t="str">
+        <v>daniel@gemartinelectrical.com</v>
+      </c>
+      <c r="C12" t="str">
+        <v>5</v>
+      </c>
+      <c r="D12" t="str">
+        <v>29</v>
+      </c>
+      <c r="E12" t="str">
+        <v>(470) 979-2061</v>
+      </c>
+      <c r="F12" t="str">
+        <v>https://blinq.me/vCWA4xO6LRTl?bs=db</v>
+      </c>
+      <c r="G12" t="str">
+        <v>https://maps.google.com/?cid=12248053110937400791&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H12" t="str">
+        <v>3870 Peachtree Industrial Blvd 340 312, Duluth, GA 30096, USA</v>
+      </c>
+      <c r="I12" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Burney Electrical Services</v>
+      </c>
+      <c r="B13" t="str">
+        <v>lburney@burneyelectricalservices.com</v>
+      </c>
+      <c r="C13" t="str">
+        <v>5</v>
+      </c>
+      <c r="D13" t="str">
+        <v>12</v>
+      </c>
+      <c r="E13" t="str">
+        <v>(404) 369-1063</v>
+      </c>
+      <c r="F13" t="str">
+        <v>https://burneyelectricalservices.com/</v>
+      </c>
+      <c r="G13" t="str">
+        <v>https://maps.google.com/?cid=4430452129245969583&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H13" t="str">
+        <v>2896 Valley Ridge Dr, Decatur, GA 30032, USA</v>
+      </c>
+      <c r="I13" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Lighthouse Electric</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Office@lighthouseelectricil.com</v>
+      </c>
+      <c r="C14" t="str">
+        <v>4.3</v>
+      </c>
+      <c r="D14" t="str">
+        <v>23</v>
+      </c>
+      <c r="E14" t="str">
+        <v>(217) 872-8808</v>
+      </c>
+      <c r="F14" t="str">
+        <v>https://www.lighthouseelectricil.com/</v>
+      </c>
+      <c r="G14" t="str">
+        <v>https://maps.google.com/?cid=1308956494112370691&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H14" t="str">
+        <v>2277 Hubbard Ave, Decatur, IL 62526, USA</v>
+      </c>
+      <c r="I14" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Hot Spot Electrical</v>
+      </c>
+      <c r="B15" t="str">
+        <v>shapiro@hotspotelectric.net</v>
+      </c>
+      <c r="C15" t="str">
+        <v>5</v>
+      </c>
+      <c r="D15" t="str">
+        <v>69</v>
+      </c>
+      <c r="E15" t="str">
+        <v>(678) 771-6085</v>
+      </c>
+      <c r="F15" t="str">
+        <v>http://hotspotelectric.net/</v>
+      </c>
+      <c r="G15" t="str">
+        <v>https://maps.google.com/?cid=5167601710071551266&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H15" t="str">
+        <v>3935 River Run Ct, Cumming, GA 30041, USA</v>
+      </c>
+      <c r="I15" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>575 electric</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Jason.mitchell@575electric.com</v>
+      </c>
+      <c r="C16" t="str">
+        <v>5</v>
+      </c>
+      <c r="D16" t="str">
+        <v>17</v>
+      </c>
+      <c r="E16" t="str">
+        <v>(404) 293-9515</v>
+      </c>
+      <c r="F16" t="str">
+        <v>https://575electric.com/</v>
+      </c>
+      <c r="G16" t="str">
+        <v>https://maps.google.com/?cid=8207680150374449049&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H16" t="str">
+        <v>1041 Boston Ridge, Woodstock, GA 30189, USA</v>
+      </c>
+      <c r="I16" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Electric Company</v>
+      </c>
+      <c r="B17" t="str">
+        <v>info@example.com</v>
+      </c>
+      <c r="C17" t="str">
+        <v>5</v>
+      </c>
+      <c r="D17" t="str">
+        <v>72</v>
+      </c>
+      <c r="E17" t="str">
+        <v>(770) 998-0060</v>
+      </c>
+      <c r="F17" t="str">
+        <v>https://electric-company.com/</v>
+      </c>
+      <c r="G17" t="str">
+        <v>https://maps.google.com/?cid=17654218059840725733&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H17" t="str">
+        <v>213 Lexington Dr, Woodstock, GA 30188, USA</v>
+      </c>
+      <c r="I17" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Blackstock Electric</v>
+      </c>
+      <c r="B18" t="str">
+        <v>da@blackstockelectric.com</v>
+      </c>
+      <c r="C18" t="str">
+        <v>4.9</v>
+      </c>
+      <c r="D18" t="str">
+        <v>83</v>
+      </c>
+      <c r="E18" t="str">
+        <v>(770) 365-5168</v>
+      </c>
+      <c r="F18" t="str">
+        <v>https://www.blackstockelectricinc.com/</v>
+      </c>
+      <c r="G18" t="str">
+        <v>https://maps.google.com/?cid=11120832181774655585&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H18" t="str">
+        <v>1010 James Burgess Rd, Suwanee, GA 30024, USA</v>
+      </c>
+      <c r="I18" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Certified Electric, Inc</v>
+      </c>
+      <c r="B19" t="str">
+        <v>dispatcher@certifiedelectric.net</v>
+      </c>
+      <c r="C19" t="str">
+        <v>4.6</v>
+      </c>
+      <c r="D19" t="str">
+        <v>71</v>
+      </c>
+      <c r="E19" t="str">
+        <v>(912) 265-3419</v>
+      </c>
+      <c r="F19" t="str">
+        <v>https://certifiedelectric.net/</v>
+      </c>
+      <c r="G19" t="str">
+        <v>https://maps.google.com/?cid=1412885056572651396&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H19" t="str">
+        <v>109 Key Dr, Brunswick, GA 31520, USA</v>
+      </c>
+      <c r="I19" t="str">
+        <v>2026-07-12</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I19"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I20"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Business Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Stars</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Reviews</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Website</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Google Maps URL</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Address</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Date Found</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>S&amp;W Plumbing</v>
+      </c>
+      <c r="B2" t="str">
+        <v>scheduling@sandwplumbing.com</v>
+      </c>
+      <c r="C2">
+        <v>4.7</v>
+      </c>
+      <c r="D2">
+        <v>82</v>
+      </c>
+      <c r="E2" t="str">
+        <v>(770) 831-7505</v>
+      </c>
+      <c r="F2" t="str">
+        <v>http://sandwplumbing.com/</v>
+      </c>
+      <c r="G2" t="str">
+        <v>https://maps.google.com/?cid=11527746932332505740&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H2" t="str">
+        <v>961 Chestnut St SE #107, Gainesville, GA 30501, USA</v>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Whitmire Plumbing &amp; Electric</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ADMIN@CALLWHITMIRE.COM</v>
+      </c>
+      <c r="C3">
+        <v>4.5</v>
+      </c>
+      <c r="D3">
+        <v>100</v>
+      </c>
+      <c r="E3" t="str">
+        <v>(770) 531-1010</v>
+      </c>
+      <c r="F3" t="str">
+        <v>https://www.callwhitmire.com/</v>
+      </c>
+      <c r="G3" t="str">
+        <v>https://maps.google.com/?cid=15542517201600839577&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H3" t="str">
+        <v>138 Clarks Bridge Rd, Gainesville, GA 30501, USA</v>
+      </c>
+      <c r="I3" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Roberts Plumbing, Inc.</v>
+      </c>
+      <c r="B4" t="str">
+        <v>%20service@callrobertsplumbing.com</v>
+      </c>
+      <c r="C4">
+        <v>4.1</v>
+      </c>
+      <c r="D4">
+        <v>49</v>
+      </c>
+      <c r="E4" t="str">
+        <v>(770) 967-1119</v>
+      </c>
+      <c r="F4" t="str">
+        <v>http://www.callrobertsplumbing.com/</v>
+      </c>
+      <c r="G4" t="str">
+        <v>https://maps.google.com/?cid=4994194242831857759&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H4" t="str">
+        <v>821 Dawsonville Hwy, Gainesville, GA 30501, USA</v>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Premier Plumbing Solutions</v>
+      </c>
+      <c r="B5" t="str">
+        <v>tim@premier-plumbing-solutions.com</v>
+      </c>
+      <c r="C5">
+        <v>4.9</v>
+      </c>
+      <c r="D5">
+        <v>124</v>
+      </c>
+      <c r="E5" t="str">
+        <v>(770) 616-8590</v>
+      </c>
+      <c r="F5" t="str">
+        <v>http://www.premier-plumbing-solutions.com/</v>
+      </c>
+      <c r="G5" t="str">
+        <v>https://maps.google.com/?cid=12345667334664111916&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H5" t="str">
+        <v>3925 Oakwood Rd, Oakwood, GA 30566, USA</v>
+      </c>
+      <c r="I5" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>A Drain Doctor plumbing llc</v>
+      </c>
+      <c r="B6" t="str">
+        <v>contact@ADrainDoctor.com</v>
+      </c>
+      <c r="C6">
+        <v>4.9</v>
+      </c>
+      <c r="D6">
+        <v>68</v>
+      </c>
+      <c r="E6" t="str">
+        <v>(706) 278-7997</v>
+      </c>
+      <c r="F6" t="str">
+        <v>https://www.adraindoctor.com/</v>
+      </c>
+      <c r="G6" t="str">
+        <v>https://maps.google.com/?cid=8957198901505259185&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H6" t="str">
+        <v>3499 Keith Vly Rd NE, Dalton, GA 30721, USA</v>
+      </c>
+      <c r="I6" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Ace Plumbing &amp; Drain Cleaning</v>
+      </c>
+      <c r="B7" t="str">
+        <v>aceplumbing.ga1@gmail.com</v>
+      </c>
+      <c r="C7">
+        <v>4.6</v>
+      </c>
+      <c r="D7">
+        <v>61</v>
+      </c>
+      <c r="E7" t="str">
+        <v>(706) 270-2276</v>
+      </c>
+      <c r="F7" t="str">
+        <v>https://aceplumbingofdalton.com/?utm_source=GP_Website&amp;utm_medium=GP</v>
+      </c>
+      <c r="G7" t="str">
+        <v>https://maps.google.com/?cid=12274968545200454038&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H7" t="str">
+        <v>3073 Five Springs Rd SE, Dalton, GA 30721, USA</v>
+      </c>
+      <c r="I7" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>A A &amp; A Drain Cleaning and Septic Tank Pumping</v>
+      </c>
+      <c r="B8" t="str">
+        <v>aaapumping09@yahoo.com</v>
+      </c>
+      <c r="C8">
+        <v>4.8</v>
+      </c>
+      <c r="D8">
+        <v>45</v>
+      </c>
+      <c r="E8" t="str">
+        <v>(706) 226-1267</v>
+      </c>
+      <c r="F8" t="str">
+        <v>http://www.aaadraincleaning.net/</v>
+      </c>
+      <c r="G8" t="str">
+        <v>https://maps.google.com/?cid=17629225242494077829&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H8" t="str">
+        <v>4133 Tibbs Bridge Rd SE, Dalton, GA 30721, USA</v>
+      </c>
+      <c r="I8" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Rapid Flow Plumbing</v>
+      </c>
+      <c r="B9" t="str">
+        <v>rapidflow@bellsouth.net</v>
+      </c>
+      <c r="C9">
+        <v>4.6</v>
+      </c>
+      <c r="D9">
+        <v>42</v>
+      </c>
+      <c r="E9" t="str">
+        <v>(770) 441-4853</v>
+      </c>
+      <c r="F9" t="str">
+        <v>http://rapidflowplumbing.com/</v>
+      </c>
+      <c r="G9" t="str">
+        <v>https://maps.google.com/?cid=8807441097767454865&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H9" t="str">
+        <v>401 Old Mill Rd Unit c, Cartersville, GA 30120, USA</v>
+      </c>
+      <c r="I9" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Beacon Plumbing Services</v>
+      </c>
+      <c r="B10" t="str">
+        <v>service@beacon-plumbing.com</v>
+      </c>
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="D10">
+        <v>17</v>
+      </c>
+      <c r="E10" t="str">
+        <v>(770) 881-6748</v>
+      </c>
+      <c r="F10" t="str">
+        <v>http://beacon-plumbing.com/</v>
+      </c>
+      <c r="G10" t="str">
+        <v>https://maps.google.com/?cid=11057949938413650837&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H10" t="str">
+        <v>23 Treemont Dr SE, Cartersville, GA 30121, USA</v>
+      </c>
+      <c r="I10" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Peach Plumbing and Water Heater</v>
+      </c>
+      <c r="B11" t="str">
+        <v>info@peachplumbingga.com</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="D11">
+        <v>41</v>
+      </c>
+      <c r="E11" t="str">
+        <v>(770) 285-0399</v>
+      </c>
+      <c r="F11" t="str">
+        <v>http://peachplumbingga.com/</v>
+      </c>
+      <c r="G11" t="str">
+        <v>https://maps.google.com/?cid=10915787145887937406&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H11" t="str">
+        <v>4357 Cobb Pkwy N, Acworth, GA 30101, USA</v>
+      </c>
+      <c r="I11" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Westgate Plumbing Services</v>
+      </c>
+      <c r="B12" t="str">
+        <v>dummytext@gmail.com</v>
+      </c>
+      <c r="C12">
+        <v>5</v>
+      </c>
+      <c r="D12">
+        <v>27</v>
+      </c>
+      <c r="E12" t="str">
+        <v>(762) 265-9092</v>
+      </c>
+      <c r="F12" t="str">
+        <v>https://westgateplumbingservices.com/rome-ga/</v>
+      </c>
+      <c r="G12" t="str">
+        <v>https://maps.google.com/?cid=1165815836092574369&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H12" t="str">
+        <v>901 N Broad St #213, Rome, GA 30161, USA</v>
+      </c>
+      <c r="I12" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Clay Henderson Plumbing, Inc.</v>
+      </c>
+      <c r="B13" t="str">
+        <v>clayhendersonplumbing@gmail.com</v>
+      </c>
+      <c r="C13">
+        <v>4.9</v>
+      </c>
+      <c r="D13">
+        <v>33</v>
+      </c>
+      <c r="E13" t="str">
+        <v>(706) 767-2499</v>
+      </c>
+      <c r="F13" t="str">
+        <v>http://www.clayhendersonplumbing.net/</v>
+      </c>
+      <c r="G13" t="str">
+        <v>https://maps.google.com/?cid=18382890320127631224&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H13" t="str">
+        <v>414 McClain Rd, Kingston, GA 30145, USA</v>
+      </c>
+      <c r="I13" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>On Point Plumbing</v>
+      </c>
+      <c r="B14" t="str">
+        <v>onpointplumbing65@gmail.com</v>
+      </c>
+      <c r="C14">
+        <v>5</v>
+      </c>
+      <c r="D14">
+        <v>12</v>
+      </c>
+      <c r="E14" t="str">
+        <v>(770) 880-0065</v>
+      </c>
+      <c r="F14" t="str">
+        <v>https://onpointplumbingga.com/?utm_source=google&amp;utm_medium=biz-profile&amp;utm_campaign=gbp-main</v>
+      </c>
+      <c r="G14" t="str">
+        <v>https://maps.google.com/?cid=68331225346960309&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H14" t="str">
+        <v>309 Oak Hill Ln, Canton, GA 30115, USA</v>
+      </c>
+      <c r="I14" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Odds and Ends Plumbing</v>
+      </c>
+      <c r="B15" t="str">
+        <v>example@mail.com</v>
+      </c>
+      <c r="C15">
+        <v>5</v>
+      </c>
+      <c r="D15">
+        <v>60</v>
+      </c>
+      <c r="E15" t="str">
+        <v>(770) 301-6317</v>
+      </c>
+      <c r="F15" t="str">
+        <v>https://www.oddsandendsplumbing.com/</v>
+      </c>
+      <c r="G15" t="str">
+        <v>https://maps.google.com/?cid=8119039356587974547&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H15" t="str">
+        <v>10 1/2 Greenville St S, Newnan, GA 30263, USA</v>
+      </c>
+      <c r="I15" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Parker's Plumbing</v>
+      </c>
+      <c r="B16" t="str">
+        <v>service@parkersplumbing.com</v>
+      </c>
+      <c r="C16">
+        <v>4.8</v>
+      </c>
+      <c r="D16">
+        <v>19</v>
+      </c>
+      <c r="E16" t="str">
+        <v>(770) 251-5172</v>
+      </c>
+      <c r="F16" t="str">
+        <v>https://www.parkersplumbing.com/</v>
+      </c>
+      <c r="G16" t="str">
+        <v>https://maps.google.com/?cid=16245227226363162057&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H16" t="str">
+        <v>200 W Ct Square, Newnan, GA 30263, USA</v>
+      </c>
+      <c r="I16" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>GoRapid Inc.</v>
+      </c>
+      <c r="B17" t="str">
+        <v>jacob@gorapid.us</v>
+      </c>
+      <c r="C17">
+        <v>4.6</v>
+      </c>
+      <c r="D17">
+        <v>93</v>
+      </c>
+      <c r="E17" t="str">
+        <v>(770) 883-3997</v>
+      </c>
+      <c r="F17" t="str">
+        <v>https://833gorapid.com/</v>
+      </c>
+      <c r="G17" t="str">
+        <v>https://maps.google.com/?cid=9425243411659715487&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H17" t="str">
+        <v>232 Robinson Rd, Newnan, GA 30263, USA</v>
+      </c>
+      <c r="I17" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Alliance Leak Detection</v>
+      </c>
+      <c r="B18" t="str">
+        <v>allianceleak@gmail.com</v>
+      </c>
+      <c r="C18">
+        <v>4.8</v>
+      </c>
+      <c r="D18">
+        <v>31</v>
+      </c>
+      <c r="E18" t="str">
+        <v>(770) 415-8457</v>
+      </c>
+      <c r="F18" t="str">
+        <v>https://www.allianceleak.com/</v>
+      </c>
+      <c r="G18" t="str">
+        <v>https://maps.google.com/?cid=14168303949020911770&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H18" t="str">
+        <v>1095 Raymond Hill Rd, Newnan, GA 30265, USA</v>
+      </c>
+      <c r="I18" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Davison Dependable Plumbing</v>
+      </c>
+      <c r="B19" t="str">
+        <v>info@davisondependableplumbing.com</v>
+      </c>
+      <c r="C19">
+        <v>4.7</v>
+      </c>
+      <c r="D19">
+        <v>22</v>
+      </c>
+      <c r="E19" t="str">
+        <v>(678) 423-1009</v>
+      </c>
+      <c r="F19" t="str">
+        <v>https://www.davisondependableplumbing.com/</v>
+      </c>
+      <c r="G19" t="str">
+        <v>https://maps.google.com/?cid=906726216252607981&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H19" t="str">
+        <v>152 Wallace Gray Rd, Newnan, GA 30263, USA</v>
+      </c>
+      <c r="I19" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Benjamin Franklin Plumbing Fayette-Coweta</v>
+      </c>
+      <c r="B20" t="str">
+        <v>greerplumbingenterprises@gmail.com</v>
+      </c>
+      <c r="C20">
+        <v>5</v>
+      </c>
+      <c r="D20">
+        <v>24</v>
+      </c>
+      <c r="E20" t="str">
+        <v>(470) 975-7770</v>
+      </c>
+      <c r="F20" t="str">
+        <v>https://www.benjaminfranklinplumbing.com/fayette-coweta/</v>
+      </c>
+      <c r="G20" t="str">
+        <v>https://maps.google.com/?cid=9780210981604335520&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H20" t="str">
+        <v>118 Palmetto Rd suite g, Tyrone, GA 30290, USA</v>
+      </c>
+      <c r="I20" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I20"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I26"/>
   <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="35.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
     <col min="3" max="3" width="6.83203125" customWidth="1"/>
     <col min="4" max="4" width="8.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="40.83203125" customWidth="1"/>
     <col min="7" max="7" width="50.83203125" customWidth="1"/>
-    <col min="8" max="8" width="45.83203125" customWidth="1"/>
+    <col min="8" max="8" width="50.83203125" customWidth="1"/>
     <col min="9" max="9" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1995,529 +3129,1508 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Bryan Electric, Inc.</v>
+        <v>Plumbers United, Inc.</v>
       </c>
       <c r="B2" t="str">
-        <v>info@bryanelectricinc.com</v>
-      </c>
-      <c r="C2" t="str">
-        <v>4</v>
-      </c>
-      <c r="D2" t="str">
-        <v>21</v>
+        <v>info@plumbersunited.com</v>
+      </c>
+      <c r="C2">
+        <v>4.8</v>
+      </c>
+      <c r="D2">
+        <v>39</v>
       </c>
       <c r="E2" t="str">
-        <v>(770) 680-2144</v>
+        <v>(770) 716-9900</v>
       </c>
       <c r="F2" t="str">
-        <v>http://www.bryanelectricinc.com/</v>
+        <v>https://www.plumbersunited.com/</v>
       </c>
       <c r="G2" t="str">
-        <v>https://maps.google.com/?cid=14552314039426656722&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=5668861502182525011&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H2" t="str">
-        <v>1840 Grassland Pkwy #200, Alpharetta, GA 30004, USA</v>
+        <v>131 Nail Rd, McDonough, GA 30253, USA</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>JustFixToday - Handyman Services in Alpharetta GA | Painter | Plumber | Drywall | AC Repair | Electrical Repair | Carpenter</v>
+        <v>Essential Plumbing</v>
       </c>
       <c r="B3" t="str">
-        <v>info@justfixtoday.com</v>
-      </c>
-      <c r="C3" t="str">
+        <v>Zbates5@gmail.com</v>
+      </c>
+      <c r="C3">
         <v>5</v>
       </c>
-      <c r="D3" t="str">
-        <v>135</v>
+      <c r="D3">
+        <v>18</v>
       </c>
       <c r="E3" t="str">
-        <v>(678) 549-8083</v>
+        <v>(678) 572-9848</v>
       </c>
       <c r="F3" t="str">
-        <v>https://www.justfixtoday.com/</v>
+        <v>http://www.essentialplumb.com/</v>
       </c>
       <c r="G3" t="str">
-        <v>https://maps.google.com/?cid=1787476070147627322&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=10549729453663942933&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H3" t="str">
-        <v>2425 Traywick Chase, Alpharetta, GA 30004, USA</v>
+        <v>243 Winding Way, Jackson, GA 30233, USA</v>
       </c>
       <c r="I3" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Southern Electric Co</v>
+        <v>Wells Septic and Precasting</v>
       </c>
       <c r="B4" t="str">
-        <v>controller@southernelectriccompany.com</v>
-      </c>
-      <c r="C4" t="str">
-        <v>4.2</v>
-      </c>
-      <c r="D4" t="str">
-        <v>11</v>
+        <v>2jwells2@bellsouth.net</v>
+      </c>
+      <c r="C4">
+        <v>4.5</v>
+      </c>
+      <c r="D4">
+        <v>51</v>
       </c>
       <c r="E4" t="str">
-        <v>(770) 740-9553</v>
+        <v>(770) 412-9494</v>
       </c>
       <c r="F4" t="str">
-        <v>https://southernelectriccompany.com/</v>
+        <v>https://www.wellsseptic.com/</v>
       </c>
       <c r="G4" t="str">
-        <v>https://maps.google.com/?cid=2412617203072986788&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=6570412738183082919&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H4" t="str">
-        <v>510 Winkler Dr #100, Alpharetta, GA 30004, USA</v>
+        <v>2040 Williamson Rd, Griffin, GA 30224, USA</v>
       </c>
       <c r="I4" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Sharp Electrical Contractors</v>
+        <v>ABBA &amp; MAR PLUMBING</v>
       </c>
       <c r="B5" t="str">
-        <v>impallari@gmail.com</v>
-      </c>
-      <c r="C5" t="str">
-        <v>5</v>
-      </c>
-      <c r="D5" t="str">
-        <v>12</v>
+        <v>info@abbamarplumbing.com</v>
+      </c>
+      <c r="C5">
+        <v>4.9</v>
+      </c>
+      <c r="D5">
+        <v>150</v>
       </c>
       <c r="E5" t="str">
-        <v>(678) 939-1907</v>
+        <v>(678) 712-6359</v>
       </c>
       <c r="F5" t="str">
-        <v>http://www.sharpelectricalcontractorsinc.com/</v>
+        <v>http://www.abbamarplumbing.com/</v>
       </c>
       <c r="G5" t="str">
-        <v>https://maps.google.com/?cid=15784420237876544597&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=18266005037053496787&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H5" t="str">
-        <v>4571 Oakhurst Ln, Alpharetta, GA 30004, USA</v>
+        <v>66 Chamisa Rd, Covington, GA 30016, USA</v>
       </c>
       <c r="I5" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Ray's Electrical Services, LLC.</v>
+        <v>Georgia Plumbing Pros LLC</v>
       </c>
       <c r="B6" t="str">
-        <v>ray.electric@yahoo.com</v>
-      </c>
-      <c r="C6" t="str">
-        <v>5</v>
-      </c>
-      <c r="D6" t="str">
-        <v>33</v>
+        <v>dispatcher.gpp@gmail.com</v>
+      </c>
+      <c r="C6">
+        <v>4.5</v>
+      </c>
+      <c r="D6">
+        <v>21</v>
       </c>
       <c r="E6" t="str">
-        <v>(404) 934-3725</v>
+        <v>(678) 449-5536</v>
       </c>
       <c r="F6" t="str">
-        <v>https://rayselectricalservices.net/</v>
+        <v>https://gaplumbingpros.com/</v>
       </c>
       <c r="G6" t="str">
-        <v>https://maps.google.com/?cid=17255572914718368004&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=3563862642173052505&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H6" t="str">
-        <v>11877 Douglas Rd, Johns Creek, GA 30005, USA</v>
+        <v>1055 Hanover Dr Suite B, Madison, GA 30650, USA</v>
       </c>
       <c r="I6" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>JA IT ELECTRIC</v>
+        <v>HammerTime Roofing &amp; Restoration LLC</v>
       </c>
       <c r="B7" t="str">
-        <v>contact@jaitelectric.com</v>
-      </c>
-      <c r="C7" t="str">
-        <v>4.9</v>
-      </c>
-      <c r="D7" t="str">
-        <v>79</v>
+        <v>HammerTimeRR@outlook.com</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7">
+        <v>126</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>(470) 746-8573</v>
       </c>
       <c r="F7" t="str">
-        <v>https://www.jaitelectric.com/</v>
+        <v>http://www.ht-roofing.com/</v>
       </c>
       <c r="G7" t="str">
-        <v>https://maps.google.com/?cid=16789752584030982869&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=11011728836810236649&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H7" t="str">
-        <v>3824 Dandridge Way NW, Duluth, GA 30096, USA</v>
+        <v>2135 Pace St, Covington, GA 30014, USA</v>
       </c>
       <c r="I7" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>DSL Electric</v>
+        <v>Plumbing &amp; Waterproofing Unlimited</v>
       </c>
       <c r="B8" t="str">
-        <v>dslelectric@yahoo.com</v>
-      </c>
-      <c r="C8" t="str">
+        <v>info@plumbingunlimitedga.com</v>
+      </c>
+      <c r="C8">
         <v>4.7</v>
       </c>
-      <c r="D8" t="str">
-        <v>143</v>
+      <c r="D8">
+        <v>77</v>
       </c>
       <c r="E8" t="str">
-        <v>(470) 637-2322</v>
+        <v>(404) 441-5723</v>
       </c>
       <c r="F8" t="str">
-        <v>https://www.dslelectric.net/</v>
+        <v>http://plumbingunlimitedga.com/</v>
       </c>
       <c r="G8" t="str">
-        <v>https://maps.google.com/?cid=1906140520379199906&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=9337026794714339584&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H8" t="str">
-        <v>1159 Reading Dr NW, Acworth, GA 30102, USA</v>
+        <v>2274 Salem Rd SE Ste.1061808, Conyers, GA 30013, USA</v>
       </c>
       <c r="I8" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>M.D. Contracting Solutions</v>
+        <v>Todd Young Plumbing Inc</v>
       </c>
       <c r="B9" t="str">
-        <v>admin@mdcontractingsolutions.com</v>
-      </c>
-      <c r="C9" t="str">
-        <v>5</v>
-      </c>
-      <c r="D9" t="str">
-        <v>137</v>
+        <v>quotes@toddyoungplumbing.com</v>
+      </c>
+      <c r="C9">
+        <v>2.9</v>
+      </c>
+      <c r="D9">
+        <v>16</v>
       </c>
       <c r="E9" t="str">
-        <v>(678) 636-9692</v>
+        <v>(770) 860-1005</v>
       </c>
       <c r="F9" t="str">
-        <v>https://www.mdcontractingsolutions.com/</v>
+        <v>https://www.toddyoungplumbing.com/</v>
       </c>
       <c r="G9" t="str">
-        <v>https://maps.google.com/?cid=9302632286792896560&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=1089819357759088721&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H9" t="str">
-        <v>2244 NW Pkwy SE Ste A, Marietta, GA 30067, USA</v>
+        <v>1137 Brett Dr SW, Conyers, GA 30094, USA</v>
       </c>
       <c r="I9" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>VIP Electrical Service</v>
+        <v>Apex Supply - Conyers</v>
       </c>
       <c r="B10" t="str">
-        <v>vipelservice@gmail.com</v>
-      </c>
-      <c r="C10" t="str">
-        <v>5</v>
-      </c>
-      <c r="D10" t="str">
-        <v>57</v>
+        <v>prf513@hajoca.com</v>
+      </c>
+      <c r="C10">
+        <v>4.8</v>
+      </c>
+      <c r="D10">
+        <v>11</v>
       </c>
       <c r="E10" t="str">
-        <v>(706) 510-5132</v>
+        <v>(678) 342-3121</v>
       </c>
       <c r="F10" t="str">
-        <v>http://vipelectricalservice.co/</v>
+        <v>https://apexsupplyconyers.com/</v>
       </c>
       <c r="G10" t="str">
-        <v>https://maps.google.com/?cid=5752995803636552844&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=9902393229941911207&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H10" t="str">
-        <v>3327 Club Pl, Duluth, GA 30096, USA</v>
+        <v>593 Sigman Rd NE Ste 200, Conyers, GA 30013, USA</v>
       </c>
       <c r="I10" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Alpine Electrical Solutions</v>
+        <v>PlumberATL</v>
       </c>
       <c r="B11" t="str">
-        <v>info@alpelecsolutions.com</v>
-      </c>
-      <c r="C11" t="str">
-        <v>5</v>
-      </c>
-      <c r="D11" t="str">
-        <v>14</v>
+        <v>contact@plumberatl.com</v>
+      </c>
+      <c r="C11">
+        <v>4.8</v>
+      </c>
+      <c r="D11">
+        <v>46</v>
       </c>
       <c r="E11" t="str">
-        <v>(470) 896-6060</v>
+        <v>(678) 409-2305</v>
       </c>
       <c r="F11" t="str">
-        <v>https://alpelecsolutions.com/</v>
+        <v>http://plumberatl.com/</v>
       </c>
       <c r="G11" t="str">
-        <v>https://maps.google.com/?cid=5558601400349421621&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=17634784513518447059&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H11" t="str">
-        <v>3675 Crestwood Pkwy NW #400, Duluth, GA 30096, USA</v>
+        <v>6110 GA-20, Loganville, GA 30052, USA</v>
       </c>
       <c r="I11" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>GE Martin Electrical LLC</v>
+        <v>Bulldog Plumbing Company</v>
       </c>
       <c r="B12" t="str">
-        <v>daniel@gemartinelectrical.com</v>
-      </c>
-      <c r="C12" t="str">
-        <v>5</v>
-      </c>
-      <c r="D12" t="str">
-        <v>29</v>
+        <v>bulldog.plumbing@yahoo.com</v>
+      </c>
+      <c r="C12">
+        <v>4.8</v>
+      </c>
+      <c r="D12">
+        <v>118</v>
       </c>
       <c r="E12" t="str">
-        <v>(470) 979-2061</v>
+        <v>(404) 787-3175</v>
       </c>
       <c r="F12" t="str">
-        <v>https://blinq.me/vCWA4xO6LRTl?bs=db</v>
+        <v>http://www.bulldogplumbing.net/</v>
       </c>
       <c r="G12" t="str">
-        <v>https://maps.google.com/?cid=12248053110937400791&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=1602670210935310613&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H12" t="str">
-        <v>3870 Peachtree Industrial Blvd 340 312, Duluth, GA 30096, USA</v>
+        <v>512 Grayson Pkwy, Grayson, GA 30017, USA</v>
       </c>
       <c r="I12" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Burney Electrical Services</v>
+        <v>Leak Detection Service Pros</v>
       </c>
       <c r="B13" t="str">
-        <v>lburney@burneyelectricalservices.com</v>
-      </c>
-      <c r="C13" t="str">
+        <v>leakdsp@gmail.com</v>
+      </c>
+      <c r="C13">
         <v>5</v>
       </c>
-      <c r="D13" t="str">
-        <v>12</v>
+      <c r="D13">
+        <v>34</v>
       </c>
       <c r="E13" t="str">
-        <v>(404) 369-1063</v>
+        <v>(678) 238-5414</v>
       </c>
       <c r="F13" t="str">
-        <v>https://burneyelectricalservices.com/</v>
+        <v>https://leakdetectionsp.com/</v>
       </c>
       <c r="G13" t="str">
-        <v>https://maps.google.com/?cid=4430452129245969583&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=3495103423133090906&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H13" t="str">
-        <v>2896 Valley Ridge Dr, Decatur, GA 30032, USA</v>
+        <v>2330 Scenic Hwy S #225, Snellville, GA 30078, USA</v>
       </c>
       <c r="I13" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Lighthouse Electric</v>
+        <v>Nick-Plumbing Inc.</v>
       </c>
       <c r="B14" t="str">
-        <v>Office@lighthouseelectricil.com</v>
-      </c>
-      <c r="C14" t="str">
-        <v>4.3</v>
-      </c>
-      <c r="D14" t="str">
-        <v>23</v>
+        <v>nick.plumbing@yahoo.com</v>
+      </c>
+      <c r="C14">
+        <v>4.9</v>
+      </c>
+      <c r="D14">
+        <v>34</v>
       </c>
       <c r="E14" t="str">
-        <v>(217) 872-8808</v>
+        <v>(404) 604-4619</v>
       </c>
       <c r="F14" t="str">
-        <v>https://www.lighthouseelectricil.com/</v>
+        <v>http://nick-plumbing.com/</v>
       </c>
       <c r="G14" t="str">
-        <v>https://maps.google.com/?cid=1308956494112370691&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=12439027872372117987&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H14" t="str">
-        <v>2277 Hubbard Ave, Decatur, IL 62526, USA</v>
+        <v>1000 Peachtree Industrial Blvd Ste 6-388, Suwanee, GA 30024, USA</v>
       </c>
       <c r="I14" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Hot Spot Electrical</v>
+        <v>All Advance Services</v>
       </c>
       <c r="B15" t="str">
-        <v>shapiro@hotspotelectric.net</v>
-      </c>
-      <c r="C15" t="str">
-        <v>5</v>
-      </c>
-      <c r="D15" t="str">
-        <v>69</v>
+        <v>chally@alladvanceservice.com</v>
+      </c>
+      <c r="C15">
+        <v>4.8</v>
+      </c>
+      <c r="D15">
+        <v>45</v>
       </c>
       <c r="E15" t="str">
-        <v>(678) 771-6085</v>
+        <v>(770) 274-6265</v>
       </c>
       <c r="F15" t="str">
-        <v>http://hotspotelectric.net/</v>
+        <v>http://alladvanceservice.com/</v>
       </c>
       <c r="G15" t="str">
-        <v>https://maps.google.com/?cid=5167601710071551266&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=3378199229948399419&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H15" t="str">
-        <v>3935 River Run Ct, Cumming, GA 30041, USA</v>
+        <v>3947 Lawrenceville-Suwanee Rd, Suwanee, GA 30024, USA</v>
       </c>
       <c r="I15" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>575 electric</v>
+        <v>FIX-R-US</v>
       </c>
       <c r="B16" t="str">
-        <v>Jason.mitchell@575electric.com</v>
-      </c>
-      <c r="C16" t="str">
-        <v>5</v>
-      </c>
-      <c r="D16" t="str">
-        <v>17</v>
+        <v>info@fixrus.com</v>
+      </c>
+      <c r="C16">
+        <v>4.6</v>
+      </c>
+      <c r="D16">
+        <v>56</v>
       </c>
       <c r="E16" t="str">
-        <v>(404) 293-9515</v>
+        <v>(678) 719-9900</v>
       </c>
       <c r="F16" t="str">
-        <v>https://575electric.com/</v>
+        <v>https://www.fixrus.com/</v>
       </c>
       <c r="G16" t="str">
-        <v>https://maps.google.com/?cid=8207680150374449049&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=10841415379020398729&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H16" t="str">
-        <v>1041 Boston Ridge, Woodstock, GA 30189, USA</v>
+        <v>3947 Lawrenceville-Suwanee Rd Ste A, Suwanee, GA 30024, USA</v>
       </c>
       <c r="I16" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Electric Company</v>
+        <v>Mulberry Plumbing Services</v>
       </c>
       <c r="B17" t="str">
-        <v>info@example.com</v>
-      </c>
-      <c r="C17" t="str">
+        <v>mulberryplumbingservices@gmail.com</v>
+      </c>
+      <c r="C17">
         <v>5</v>
       </c>
-      <c r="D17" t="str">
-        <v>72</v>
+      <c r="D17">
+        <v>29</v>
       </c>
       <c r="E17" t="str">
-        <v>(770) 998-0060</v>
+        <v>(770) 744-1880</v>
       </c>
       <c r="F17" t="str">
-        <v>https://electric-company.com/</v>
+        <v>https://www.mulberryplumbingservices.com/</v>
       </c>
       <c r="G17" t="str">
-        <v>https://maps.google.com/?cid=17654218059840725733&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=2327746073260919084&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H17" t="str">
-        <v>213 Lexington Dr, Woodstock, GA 30188, USA</v>
+        <v>4992 B U Bowman Dr Ste 104, Buford, GA 30518, USA</v>
       </c>
       <c r="I17" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Blackstock Electric</v>
+        <v>Cornerstone Plumbing &amp; Mechanical LLC</v>
       </c>
       <c r="B18" t="str">
-        <v>da@blackstockelectric.com</v>
-      </c>
-      <c r="C18" t="str">
+        <v>michael@cstonepm.com</v>
+      </c>
+      <c r="C18">
         <v>4.9</v>
       </c>
-      <c r="D18" t="str">
-        <v>83</v>
+      <c r="D18">
+        <v>122</v>
       </c>
       <c r="E18" t="str">
-        <v>(770) 365-5168</v>
+        <v>(404) 569-5687</v>
       </c>
       <c r="F18" t="str">
-        <v>https://www.blackstockelectricinc.com/</v>
+        <v>https://cornerstoneplumbingga.com/</v>
       </c>
       <c r="G18" t="str">
-        <v>https://maps.google.com/?cid=11120832181774655585&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+        <v>https://maps.google.com/?cid=13501579207528860665&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
       </c>
       <c r="H18" t="str">
-        <v>1010 James Burgess Rd, Suwanee, GA 30024, USA</v>
+        <v>4152 Clark Hill Ct NE, Buford, GA 30519, USA</v>
       </c>
       <c r="I18" t="str">
-        <v>2026-07-12</v>
+        <v>2026-07-14</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Certified Electric, Inc</v>
+        <v>Servant Plumbing of North Atlanta</v>
       </c>
       <c r="B19" t="str">
-        <v>dispatcher@certifiedelectric.net</v>
-      </c>
-      <c r="C19" t="str">
+        <v>info@servantplumbing.com</v>
+      </c>
+      <c r="C19">
+        <v>5</v>
+      </c>
+      <c r="D19">
+        <v>50</v>
+      </c>
+      <c r="E19" t="str">
+        <v>(470) 573-6944</v>
+      </c>
+      <c r="F19" t="str">
+        <v>https://servantplumbingatl.com/?utm_source=Google+&amp;utm_medium=Organic&amp;utm_campaign=gbp</v>
+      </c>
+      <c r="G19" t="str">
+        <v>https://maps.google.com/?cid=7208126319626468624&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H19" t="str">
+        <v>115 E Main St NE Suite A1B, Buford, GA 30518, USA</v>
+      </c>
+      <c r="I19" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Sloggy Plumbing</v>
+      </c>
+      <c r="B20" t="str">
+        <v>example@domain.com</v>
+      </c>
+      <c r="C20">
         <v>4.6</v>
       </c>
-      <c r="D19" t="str">
-        <v>71</v>
-      </c>
-      <c r="E19" t="str">
-        <v>(912) 265-3419</v>
-      </c>
-      <c r="F19" t="str">
-        <v>https://certifiedelectric.net/</v>
-      </c>
-      <c r="G19" t="str">
-        <v>https://maps.google.com/?cid=1412885056572651396&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
-      </c>
-      <c r="H19" t="str">
-        <v>109 Key Dr, Brunswick, GA 31520, USA</v>
-      </c>
-      <c r="I19" t="str">
-        <v>2026-07-12</v>
+      <c r="D20">
+        <v>51</v>
+      </c>
+      <c r="E20" t="str">
+        <v>(770) 231-3355</v>
+      </c>
+      <c r="F20" t="str">
+        <v>https://www.patriotservicega.com/</v>
+      </c>
+      <c r="G20" t="str">
+        <v>https://maps.google.com/?cid=10157469563444553770&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H20" t="str">
+        <v>6165 New Bethany Rd, Buford, GA 30518, USA</v>
+      </c>
+      <c r="I20" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>C&amp;A Johnson Plumbing Service LLC</v>
+      </c>
+      <c r="B21" t="str">
+        <v>eben@eyebytes.com</v>
+      </c>
+      <c r="C21">
+        <v>4.8</v>
+      </c>
+      <c r="D21">
+        <v>30</v>
+      </c>
+      <c r="E21" t="str">
+        <v>(678) 714-7814</v>
+      </c>
+      <c r="F21" t="str">
+        <v>https://cajplumbing.com/</v>
+      </c>
+      <c r="G21" t="str">
+        <v>https://maps.google.com/?cid=10461404698754667353&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H21" t="str">
+        <v>3851 Bream Ct, Buford, GA 30519, USA</v>
+      </c>
+      <c r="I21" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>G2 Plumbing Services LLC</v>
+      </c>
+      <c r="B22" t="str">
+        <v>team@latofonts.com</v>
+      </c>
+      <c r="C22">
+        <v>4.9</v>
+      </c>
+      <c r="D22">
+        <v>36</v>
+      </c>
+      <c r="E22" t="str">
+        <v>(678) 457-6512</v>
+      </c>
+      <c r="F22" t="str">
+        <v>https://g2plumbingservices.com/</v>
+      </c>
+      <c r="G22" t="str">
+        <v>https://maps.google.com/?cid=2725065276958452010&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Dacula Rd, Dacula, GA 30019, USA</v>
+      </c>
+      <c r="I22" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Millennial Plumbing &amp; Tankless</v>
+      </c>
+      <c r="B23" t="str">
+        <v>millennialplumbingandtankless@gmail.com</v>
+      </c>
+      <c r="C23">
+        <v>5</v>
+      </c>
+      <c r="D23">
+        <v>33</v>
+      </c>
+      <c r="E23" t="str">
+        <v>(470) 727-6292</v>
+      </c>
+      <c r="F23" t="str">
+        <v>https://www.millennialplumbingandtankless.com/?utm_source=gmb&amp;utm_medium=listing&amp;utm_campaign=local</v>
+      </c>
+      <c r="G23" t="str">
+        <v>https://maps.google.com/?cid=520787479516172373&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H23" t="str">
+        <v>1661 Greyleaf Ln SE, Dacula, GA 30019, USA</v>
+      </c>
+      <c r="I23" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Value Plumbing, Inc.</v>
+      </c>
+      <c r="B24" t="str">
+        <v>valueplumbinginc@gmail.com</v>
+      </c>
+      <c r="C24">
+        <v>4.9</v>
+      </c>
+      <c r="D24">
+        <v>108</v>
+      </c>
+      <c r="E24" t="str">
+        <v>(678) 725-3037</v>
+      </c>
+      <c r="F24" t="str">
+        <v>http://valueplumbinginc.com/</v>
+      </c>
+      <c r="G24" t="str">
+        <v>https://maps.google.com/?cid=9239627556401116572&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H24" t="str">
+        <v>1367 Mountain Lake Dr, Auburn, GA 30011, USA</v>
+      </c>
+      <c r="I24" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>SHARP Improvements LLC</v>
+      </c>
+      <c r="B25" t="str">
+        <v>sharpimprovementsplumbing@gmail.com</v>
+      </c>
+      <c r="C25">
+        <v>4.5</v>
+      </c>
+      <c r="D25">
+        <v>85</v>
+      </c>
+      <c r="E25" t="str">
+        <v>(404) 543-8319</v>
+      </c>
+      <c r="F25" t="str">
+        <v>https://www.sharp-improvements.com/</v>
+      </c>
+      <c r="G25" t="str">
+        <v>https://maps.google.com/?cid=8318091740610346527&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H25" t="str">
+        <v>107 Vine St Ste A, Monroe, GA 30655, USA</v>
+      </c>
+      <c r="I25" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Leader Plumbing</v>
+      </c>
+      <c r="B26" t="str">
+        <v>leaderplumbing1@gmail.com</v>
+      </c>
+      <c r="C26">
+        <v>4.8</v>
+      </c>
+      <c r="D26">
+        <v>19</v>
+      </c>
+      <c r="E26" t="str">
+        <v>(770) 266-0002</v>
+      </c>
+      <c r="F26" t="str">
+        <v>http://www.leaderplumbing.net/</v>
+      </c>
+      <c r="G26" t="str">
+        <v>https://maps.google.com/?cid=13576563045012225435&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H26" t="str">
+        <v>1550 GA-138, Monroe, GA 30655, USA</v>
+      </c>
+      <c r="I26" t="str">
+        <v>2026-07-14</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I26"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I26"/>
+  <cols>
+    <col min="1" max="1" width="35.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="6.83203125" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="40.83203125" customWidth="1"/>
+    <col min="7" max="7" width="50.83203125" customWidth="1"/>
+    <col min="8" max="8" width="50.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Business Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Stars</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Reviews</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Website</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Google Maps URL</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Address</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Date Found</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>DNA Plumbing</v>
+      </c>
+      <c r="B2" t="str">
+        <v>dnaplumbingatlanta@gmail.com</v>
+      </c>
+      <c r="C2">
+        <v>5</v>
+      </c>
+      <c r="D2">
+        <v>73</v>
+      </c>
+      <c r="E2" t="str">
+        <v>(770) 362-2238</v>
+      </c>
+      <c r="F2" t="str">
+        <v>https://dnaplumbingatlanta.com/</v>
+      </c>
+      <c r="G2" t="str">
+        <v>https://maps.google.com/?cid=2281866740697687424&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H2" t="str">
+        <v>57 Huckleberry Ln, Winder, GA 30680, USA</v>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Garner Plumbing Services</v>
+      </c>
+      <c r="B3" t="str">
+        <v>amanda@garnerplumbinginc.com</v>
+      </c>
+      <c r="C3">
+        <v>4.4</v>
+      </c>
+      <c r="D3">
+        <v>85</v>
+      </c>
+      <c r="E3" t="str">
+        <v>(706) 658-4236</v>
+      </c>
+      <c r="F3" t="str">
+        <v>https://www.garnerplumbinginc.com/?utm_source=google&amp;utm_medium=organic&amp;utm_campaign=gmb</v>
+      </c>
+      <c r="G3" t="str">
+        <v>https://maps.google.com/?cid=15032155862959102238&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H3" t="str">
+        <v>741 W Winder Industrial Pkwy, Winder, GA 30680, USA</v>
+      </c>
+      <c r="I3" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Wrench Works Plumbing</v>
+      </c>
+      <c r="B4" t="str">
+        <v>wrenchworksplumbing@hotmail.com</v>
+      </c>
+      <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4">
+        <v>57</v>
+      </c>
+      <c r="E4" t="str">
+        <v>(706) 399-6224</v>
+      </c>
+      <c r="F4" t="str">
+        <v>https://wrenchworksplumbing.com/</v>
+      </c>
+      <c r="G4" t="str">
+        <v>https://maps.google.com/?cid=15176590971418578389&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H4" t="str">
+        <v>161 Pine Rock Rd, Winder, GA 30680, USA</v>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Jefferson Plumbing Company</v>
+      </c>
+      <c r="B5" t="str">
+        <v>jeffersonplumbingco@outlook.com</v>
+      </c>
+      <c r="C5">
+        <v>4.7</v>
+      </c>
+      <c r="D5">
+        <v>96</v>
+      </c>
+      <c r="E5" t="str">
+        <v>(706) 367-5026</v>
+      </c>
+      <c r="F5" t="str">
+        <v>https://www.jeffersonplumbingco.com/</v>
+      </c>
+      <c r="G5" t="str">
+        <v>https://maps.google.com/?cid=2828315420985520293&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H5" t="str">
+        <v>167 Apex Dr suite 300, Jefferson, GA 30549, USA</v>
+      </c>
+      <c r="I5" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Gen3 Plumbing</v>
+      </c>
+      <c r="B6" t="str">
+        <v>info@gen3plumb.com</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>66</v>
+      </c>
+      <c r="E6" t="str">
+        <v>(706) 389-9679</v>
+      </c>
+      <c r="F6" t="str">
+        <v>https://www.gen3plumb.com/</v>
+      </c>
+      <c r="G6" t="str">
+        <v>https://maps.google.com/?cid=11284706629037799457&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H6" t="str">
+        <v>1395 Ronald Reagan Ln, Jefferson, GA 30549, USA</v>
+      </c>
+      <c r="I6" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>The Bliss Fix</v>
+      </c>
+      <c r="B7" t="str">
+        <v>theblissfix1@gmail.com</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7">
+        <v>105</v>
+      </c>
+      <c r="E7" t="str">
+        <v>(770) 527-9959</v>
+      </c>
+      <c r="F7" t="str">
+        <v>http://theblissfix.com/</v>
+      </c>
+      <c r="G7" t="str">
+        <v>https://maps.google.com/?cid=1155117733387859279&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Jackson Trail Rd, Jefferson, GA 30549, USA</v>
+      </c>
+      <c r="I7" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Top Tier Restoration Services</v>
+      </c>
+      <c r="B8" t="str">
+        <v>wfarmer@ttr-rs.com</v>
+      </c>
+      <c r="C8">
+        <v>4.8</v>
+      </c>
+      <c r="D8">
+        <v>21</v>
+      </c>
+      <c r="E8" t="str">
+        <v>(706) 870-0957</v>
+      </c>
+      <c r="F8" t="str">
+        <v>https://toptierrestorationservices.com/</v>
+      </c>
+      <c r="G8" t="str">
+        <v>https://maps.google.com/?cid=16332656710052972526&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H8" t="str">
+        <v>1851 Athens Hwy Unit 205, Jefferson, GA 30549, USA</v>
+      </c>
+      <c r="I8" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>North Georgia Plumbing</v>
+      </c>
+      <c r="B9" t="str">
+        <v>info@northgaplumbing.com</v>
+      </c>
+      <c r="C9">
+        <v>4.2</v>
+      </c>
+      <c r="D9">
+        <v>37</v>
+      </c>
+      <c r="E9" t="str">
+        <v>(706) 776-1499</v>
+      </c>
+      <c r="F9" t="str">
+        <v>http://www.northgaplumbing.com/</v>
+      </c>
+      <c r="G9" t="str">
+        <v>https://maps.google.com/?cid=68240513764709427&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H9" t="str">
+        <v>571 E Currahee St, Toccoa, GA 30577, USA</v>
+      </c>
+      <c r="I9" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Phillips Plumbing, Wells and Septic</v>
+      </c>
+      <c r="B10" t="str">
+        <v>phillipsapplianceandplumbing@gmail.com</v>
+      </c>
+      <c r="C10">
+        <v>4.9</v>
+      </c>
+      <c r="D10">
+        <v>119</v>
+      </c>
+      <c r="E10" t="str">
+        <v>(706) 920-4264</v>
+      </c>
+      <c r="F10" t="str">
+        <v>https://phillipsplumbing.us/</v>
+      </c>
+      <c r="G10" t="str">
+        <v>https://maps.google.com/?cid=2053676004999121567&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H10" t="str">
+        <v>471 Fred King Rd, Hartwell, GA 30643, USA</v>
+      </c>
+      <c r="I10" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>LL Grimes Plumbing</v>
+      </c>
+      <c r="B11" t="str">
+        <v>service@llgrimesplumbing.com</v>
+      </c>
+      <c r="C11">
+        <v>4.4</v>
+      </c>
+      <c r="D11">
+        <v>126</v>
+      </c>
+      <c r="E11" t="str">
+        <v>(478) 452-9175</v>
+      </c>
+      <c r="F11" t="str">
+        <v>https://llgrimes.com/</v>
+      </c>
+      <c r="G11" t="str">
+        <v>https://maps.google.com/?cid=2925954010291509390&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H11" t="str">
+        <v>149 Roberson Mill Rd, Milledgeville, GA 31061, USA</v>
+      </c>
+      <c r="I11" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>LAV Plumbing</v>
+      </c>
+      <c r="B12" t="str">
+        <v>lavplumbing@gmail.com</v>
+      </c>
+      <c r="C12">
+        <v>4.3</v>
+      </c>
+      <c r="D12">
+        <v>24</v>
+      </c>
+      <c r="E12" t="str">
+        <v>(478) 414-7791</v>
+      </c>
+      <c r="F12" t="str">
+        <v>http://lavplumbing.com/</v>
+      </c>
+      <c r="G12" t="str">
+        <v>https://maps.google.com/?cid=1019203968364467019&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2941 N Columbia St, Milledgeville, GA 31061, USA</v>
+      </c>
+      <c r="I12" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Two Brothers Handyman Services,LLC</v>
+      </c>
+      <c r="B13" t="str">
+        <v>contact@sansoxygen.com</v>
+      </c>
+      <c r="C13">
+        <v>4.8</v>
+      </c>
+      <c r="D13">
+        <v>19</v>
+      </c>
+      <c r="E13" t="str">
+        <v>(478) 804-1620</v>
+      </c>
+      <c r="F13" t="str">
+        <v>http://twobrothers31031.com/</v>
+      </c>
+      <c r="G13" t="str">
+        <v>https://maps.google.com/?cid=12017358222490515709&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H13" t="str">
+        <v>120 Crestwood Dr, Gordon, GA 31031, USA</v>
+      </c>
+      <c r="I13" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Martin's Septic Service</v>
+      </c>
+      <c r="B14" t="str">
+        <v>martinintegrity@hotmail.com</v>
+      </c>
+      <c r="C14">
+        <v>4.8</v>
+      </c>
+      <c r="D14">
+        <v>26</v>
+      </c>
+      <c r="E14" t="str">
+        <v>(478) 452-8272</v>
+      </c>
+      <c r="F14" t="str">
+        <v>http://martinseptictanksga.com/</v>
+      </c>
+      <c r="G14" t="str">
+        <v>https://maps.google.com/?cid=2439650747993245498&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H14" t="str">
+        <v>2851A Vinson Hwy, Milledgeville, GA 31061, USA</v>
+      </c>
+      <c r="I14" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Tindall Septic Tank LLC</v>
+      </c>
+      <c r="B15" t="str">
+        <v>swamplife76@yahoo.com</v>
+      </c>
+      <c r="C15">
+        <v>4.8</v>
+      </c>
+      <c r="D15">
+        <v>50</v>
+      </c>
+      <c r="E15" t="str">
+        <v>(478) 457-4243</v>
+      </c>
+      <c r="F15" t="str">
+        <v>http://tindallseptictank.com/</v>
+      </c>
+      <c r="G15" t="str">
+        <v>https://maps.google.com/?cid=10978266485710482465&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H15" t="str">
+        <v>219 Sinclair Marina Rd, Milledgeville, GA 31061, USA</v>
+      </c>
+      <c r="I15" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>The Plumber Guy</v>
+      </c>
+      <c r="B16" t="str">
+        <v>theplumberguy478@gmail.com</v>
+      </c>
+      <c r="C16">
+        <v>4.6</v>
+      </c>
+      <c r="D16">
+        <v>94</v>
+      </c>
+      <c r="E16" t="str">
+        <v>(478) 225-9701</v>
+      </c>
+      <c r="F16" t="str">
+        <v>http://calltheplumberguy.com/</v>
+      </c>
+      <c r="G16" t="str">
+        <v>https://maps.google.com/?cid=3073692146524118637&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H16" t="str">
+        <v>102 Industrial Way, Centerville, GA 31028, USA</v>
+      </c>
+      <c r="I16" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>1st Choice Plumbing -Byron,Ga.</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Robby@1STChoicePlumbing.biz</v>
+      </c>
+      <c r="C17">
+        <v>4.9</v>
+      </c>
+      <c r="D17">
+        <v>85</v>
+      </c>
+      <c r="E17" t="str">
+        <v>(478) 973-9127</v>
+      </c>
+      <c r="F17" t="str">
+        <v>http://www.1stchoiceplumbing.biz/</v>
+      </c>
+      <c r="G17" t="str">
+        <v>https://maps.google.com/?cid=8113952156467508049&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H17" t="str">
+        <v>128 Emerald Blvd, Byron, GA 31008, USA</v>
+      </c>
+      <c r="I17" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Ingram Plumbing Company of Perry Georgia</v>
+      </c>
+      <c r="B18" t="str">
+        <v>ingramplumbingcompany@gmail.com</v>
+      </c>
+      <c r="C18">
+        <v>4.8</v>
+      </c>
+      <c r="D18">
+        <v>31</v>
+      </c>
+      <c r="E18" t="str">
+        <v>(478) 987-9243</v>
+      </c>
+      <c r="F18" t="str">
+        <v>https://www.ingramplumbingcompany.com/</v>
+      </c>
+      <c r="G18" t="str">
+        <v>https://maps.google.com/?cid=8658593487861390795&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H18" t="str">
+        <v>104 Wimberly Rd, Hawkinsville, GA 31036, USA</v>
+      </c>
+      <c r="I18" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Guaranteed Home Repair, Inc.</v>
+      </c>
+      <c r="B19" t="str">
+        <v>FixGanow@gmail.com</v>
+      </c>
+      <c r="C19">
+        <v>4.9</v>
+      </c>
+      <c r="D19">
+        <v>145</v>
+      </c>
+      <c r="E19" t="str">
+        <v>(478) 365-1430</v>
+      </c>
+      <c r="F19" t="str">
+        <v>https://guaranteed.repair/</v>
+      </c>
+      <c r="G19" t="str">
+        <v>https://maps.google.com/?cid=8012224384597273667&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H19" t="str">
+        <v>720 Ivy Glen Dr, Perry, GA 31069, USA</v>
+      </c>
+      <c r="I19" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Southern Infrastructure Construction</v>
+      </c>
+      <c r="B20" t="str">
+        <v>southerninfrastructureconst@gmail.com</v>
+      </c>
+      <c r="C20">
+        <v>5</v>
+      </c>
+      <c r="D20">
+        <v>46</v>
+      </c>
+      <c r="E20" t="str">
+        <v>(478) 595-5753</v>
+      </c>
+      <c r="F20" t="str">
+        <v>https://www.southerninfrastructurellc.com/</v>
+      </c>
+      <c r="G20" t="str">
+        <v>https://maps.google.com/?cid=3880446214351171371&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H20" t="str">
+        <v>487 Perry Horton Rd, Adrian, GA 31002, USA</v>
+      </c>
+      <c r="I20" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Tony Perks Plumbing Inc</v>
+      </c>
+      <c r="B21" t="str">
+        <v>tperksplumbing@att.net</v>
+      </c>
+      <c r="C21">
+        <v>4.6</v>
+      </c>
+      <c r="D21">
+        <v>22</v>
+      </c>
+      <c r="E21" t="str">
+        <v>(912) 858-5251</v>
+      </c>
+      <c r="F21" t="str">
+        <v>http://www.tonyperksplumbing.com/</v>
+      </c>
+      <c r="G21" t="str">
+        <v>https://maps.google.com/?cid=17390532202632556827&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H21" t="str">
+        <v>271 Pevey Rd, Ellabell, GA 31308, USA</v>
+      </c>
+      <c r="I21" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Roscoe Laircey Co</v>
+      </c>
+      <c r="B22" t="str">
+        <v>service@roscoelaircey.com</v>
+      </c>
+      <c r="C22">
+        <v>4.9</v>
+      </c>
+      <c r="D22">
+        <v>128</v>
+      </c>
+      <c r="E22" t="str">
+        <v>(912) 764-3372</v>
+      </c>
+      <c r="F22" t="str">
+        <v>http://rlheatingandair.com/</v>
+      </c>
+      <c r="G22" t="str">
+        <v>https://maps.google.com/?cid=5638520897157949597&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H22" t="str">
+        <v>128 W Parrish St #1289, Statesboro, GA 30458, USA</v>
+      </c>
+      <c r="I22" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Scott Wells Plumbing Company</v>
+      </c>
+      <c r="B23" t="str">
+        <v>scottwellsplbg@coastalnow.net</v>
+      </c>
+      <c r="C23">
+        <v>3.9</v>
+      </c>
+      <c r="D23">
+        <v>15</v>
+      </c>
+      <c r="E23" t="str">
+        <v>(912) 369-2067</v>
+      </c>
+      <c r="F23" t="str">
+        <v>http://scottwellsplumbing.pro/</v>
+      </c>
+      <c r="G23" t="str">
+        <v>https://maps.google.com/?cid=13362099993025538065&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H23" t="str">
+        <v>281 John Wells Rd, Hinesville, GA 31313, USA</v>
+      </c>
+      <c r="I23" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Benjamin Franklin Plumbing of Savannah Metro</v>
+      </c>
+      <c r="B24" t="str">
+        <v>CSR.0783@benfranklinplumbing.com</v>
+      </c>
+      <c r="C24">
+        <v>5</v>
+      </c>
+      <c r="D24">
+        <v>17</v>
+      </c>
+      <c r="E24" t="str">
+        <v>(912) 388-9997</v>
+      </c>
+      <c r="F24" t="str">
+        <v>https://benjaminfranklinplumbing.com/savannah-metro/</v>
+      </c>
+      <c r="G24" t="str">
+        <v>https://maps.google.com/?cid=1517926889760478393&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H24" t="str">
+        <v>1744 Old Dean Forest Rd, Pooler, GA 31322, USA</v>
+      </c>
+      <c r="I24" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Gary McBride Plumbing Services Inc</v>
+      </c>
+      <c r="B25" t="str">
+        <v>info@garymcbrideplumbing.com</v>
+      </c>
+      <c r="C25">
+        <v>4.6</v>
+      </c>
+      <c r="D25">
+        <v>39</v>
+      </c>
+      <c r="E25" t="str">
+        <v>(912) 748-8000</v>
+      </c>
+      <c r="F25" t="str">
+        <v>https://www.garymcbrideplumbing.com/</v>
+      </c>
+      <c r="G25" t="str">
+        <v>https://maps.google.com/?cid=17132518681408653682&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H25" t="str">
+        <v>1209 US-80, Pooler, GA 31322, USA</v>
+      </c>
+      <c r="I25" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Tom Horne Supply Co Inc</v>
+      </c>
+      <c r="B26" t="str">
+        <v>contact@tomhornesupply.com</v>
+      </c>
+      <c r="C26">
+        <v>4.8</v>
+      </c>
+      <c r="D26">
+        <v>36</v>
+      </c>
+      <c r="E26" t="str">
+        <v>(229) 226-3031</v>
+      </c>
+      <c r="F26" t="str">
+        <v>http://www.tomhornesupply.com/</v>
+      </c>
+      <c r="G26" t="str">
+        <v>https://maps.google.com/?cid=12775731217968161997&amp;g_mp=Cidnb29nbGUubWFwcy5wbGFjZXMudjEuUGxhY2VzLlNlYXJjaFRleHQQAhgEIAA</v>
+      </c>
+      <c r="H26" t="str">
+        <v>218 W Monroe St, Thomasville, GA 31792, USA</v>
+      </c>
+      <c r="I26" t="str">
+        <v>2026-07-14</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>